<commit_message>
Fix Angsi TABLE I column mapping: Bulk/Grain density were offset
The TABLE I data rows have 6 columns (no Ka_grain data):
  Depth | Plug No. | Porosity% | Ka_bulk | Bulk_Density | Grain_Density

Previous mapping incorrectly placed Bulk_Density in Ka_grain_mD slot,
causing Grain_Density_gcc to be None for all 12 samples.
Also removed the non-existent Ka_grain_mD column from output headers.

https://claude.ai/code/session_016iSdMZ2YZ9rCiw11HkYQ7S
</commit_message>
<xml_diff>
--- a/RESULTS/Angsi1_ML_Dataset.xlsx
+++ b/RESULTS/Angsi1_ML_Dataset.xlsx
@@ -470,21 +470,21 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -515,7 +515,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Ka_grain_mD</t>
+          <t>Bulk_Density_gcc</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -525,65 +525,60 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Bulk_Density_gcc</t>
+          <t>Formation_Factor</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Formation_Factor</t>
+          <t>Sat_Exponent</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Sat_Exponent</t>
+          <t>RQI</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>RQI</t>
+          <t>log10_Ka</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>log10_Ka</t>
+          <t>Pc_entry_psi_Run1</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Pc_entry_psi_Run1</t>
+          <t>Sw_at_Pc_entry_Run1</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Sw_at_Pc_entry_Run1</t>
+          <t>Pc_max_psi_Run1</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Pc_max_psi_Run1</t>
+          <t>Sw_at_Pc_max_Run1</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Sw_at_Pc_max_Run1</t>
+          <t>Pc_entry_psi_Run2</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Pc_entry_psi_Run2</t>
+          <t>Sw_at_Pc_entry_Run2</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Sw_at_Pc_entry_Run2</t>
+          <t>Pc_max_psi_Run2</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Pc_max_psi_Run2</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Sw_at_Pc_max_Run2</t>
         </is>
@@ -612,22 +607,22 @@
       <c r="F2" s="2" t="n">
         <v>2.23</v>
       </c>
-      <c r="G2" s="2" t="n"/>
+      <c r="G2" s="2" t="n">
+        <v>2.66</v>
+      </c>
       <c r="H2" s="2" t="n">
-        <v>2.66</v>
+        <v>42.8</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>42.8</v>
+        <v>2.11</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>2.11</v>
+        <v>0.1635</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>0.1635</v>
-      </c>
-      <c r="L2" s="2" t="n">
         <v>0.6454</v>
       </c>
+      <c r="L2" s="2" t="n"/>
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n"/>
@@ -660,22 +655,22 @@
       <c r="F3" s="3" t="n">
         <v>2.3</v>
       </c>
-      <c r="G3" s="3" t="n"/>
+      <c r="G3" s="3" t="n">
+        <v>2.68</v>
+      </c>
       <c r="H3" s="3" t="n">
-        <v>2.68</v>
+        <v>58.03</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>58.03</v>
+        <v>2.01</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>2.01</v>
+        <v>0.1309</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>0.1309</v>
-      </c>
-      <c r="L3" s="3" t="n">
         <v>0.3892</v>
       </c>
+      <c r="L3" s="3" t="n"/>
       <c r="M3" s="3" t="n"/>
       <c r="N3" s="3" t="n"/>
       <c r="O3" s="3" t="n"/>
@@ -708,18 +703,18 @@
       <c r="F4" s="2" t="n">
         <v>2.23</v>
       </c>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>2.66</v>
       </c>
+      <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
+      <c r="J4" s="2" t="n">
+        <v>0.3436</v>
+      </c>
       <c r="K4" s="2" t="n">
-        <v>0.3436</v>
-      </c>
-      <c r="L4" s="2" t="n">
         <v>1.2878</v>
       </c>
+      <c r="L4" s="2" t="n"/>
       <c r="M4" s="2" t="n">
         <v>2.4</v>
       </c>
@@ -768,18 +763,18 @@
       <c r="F5" s="3" t="n">
         <v>2.26</v>
       </c>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n">
+      <c r="G5" s="3" t="n">
         <v>2.67</v>
       </c>
+      <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
+      <c r="J5" s="3" t="n">
+        <v>0.2262</v>
+      </c>
       <c r="K5" s="3" t="n">
-        <v>0.2262</v>
-      </c>
-      <c r="L5" s="3" t="n">
         <v>0.9025</v>
       </c>
+      <c r="L5" s="3" t="n"/>
       <c r="M5" s="3" t="n"/>
       <c r="N5" s="3" t="n"/>
       <c r="O5" s="3" t="n"/>
@@ -812,22 +807,22 @@
       <c r="F6" s="2" t="n">
         <v>2.44</v>
       </c>
-      <c r="G6" s="2" t="n"/>
+      <c r="G6" s="2" t="n">
+        <v>2.69</v>
+      </c>
       <c r="H6" s="2" t="n">
-        <v>2.69</v>
+        <v>137.6</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>137.6</v>
+        <v>1.94</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>1.94</v>
+        <v>0.0322</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>0.0322</v>
-      </c>
-      <c r="L6" s="2" t="n">
         <v>-1</v>
       </c>
+      <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="n"/>
@@ -860,18 +855,18 @@
       <c r="F7" s="3" t="n">
         <v>2.3</v>
       </c>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n">
+      <c r="G7" s="3" t="n">
         <v>2.69</v>
       </c>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
+      <c r="J7" s="3" t="n">
+        <v>0.2041</v>
+      </c>
       <c r="K7" s="3" t="n">
-        <v>0.2041</v>
-      </c>
-      <c r="L7" s="3" t="n">
         <v>0.7782</v>
       </c>
+      <c r="L7" s="3" t="n"/>
       <c r="M7" s="3" t="n"/>
       <c r="N7" s="3" t="n"/>
       <c r="O7" s="3" t="n"/>
@@ -904,18 +899,18 @@
       <c r="F8" s="2" t="n">
         <v>2.22</v>
       </c>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>2.67</v>
       </c>
+      <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
+      <c r="J8" s="2" t="n">
+        <v>0.5396</v>
+      </c>
       <c r="K8" s="2" t="n">
-        <v>0.5396</v>
-      </c>
-      <c r="L8" s="2" t="n">
         <v>1.7007</v>
       </c>
+      <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
@@ -948,18 +943,18 @@
       <c r="F9" s="3" t="n">
         <v>2.28</v>
       </c>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n">
+      <c r="G9" s="3" t="n">
         <v>2.68</v>
       </c>
+      <c r="H9" s="3" t="n"/>
       <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
+      <c r="J9" s="3" t="n">
+        <v>0.3927</v>
+      </c>
       <c r="K9" s="3" t="n">
-        <v>0.3927</v>
-      </c>
-      <c r="L9" s="3" t="n">
         <v>1.3674</v>
       </c>
+      <c r="L9" s="3" t="n"/>
       <c r="M9" s="3" t="n"/>
       <c r="N9" s="3" t="n"/>
       <c r="O9" s="3" t="n"/>
@@ -992,18 +987,18 @@
       <c r="F10" s="2" t="n">
         <v>2.3</v>
       </c>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>2.68</v>
       </c>
+      <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
+      <c r="J10" s="2" t="n">
+        <v>0.2506</v>
+      </c>
       <c r="K10" s="2" t="n">
-        <v>0.2506</v>
-      </c>
-      <c r="L10" s="2" t="n">
         <v>0.9624</v>
       </c>
+      <c r="L10" s="2" t="n"/>
       <c r="M10" s="2" t="n">
         <v>3</v>
       </c>
@@ -1052,18 +1047,18 @@
       <c r="F11" s="3" t="n">
         <v>2.24</v>
       </c>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n">
+      <c r="G11" s="3" t="n">
         <v>2.56</v>
       </c>
+      <c r="H11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
+      <c r="J11" s="3" t="n">
+        <v>0.5668</v>
+      </c>
       <c r="K11" s="3" t="n">
-        <v>0.5668</v>
-      </c>
-      <c r="L11" s="3" t="n">
         <v>1.7143</v>
       </c>
+      <c r="L11" s="3" t="n"/>
       <c r="M11" s="3" t="n"/>
       <c r="N11" s="3" t="n"/>
       <c r="O11" s="3" t="n"/>
@@ -1096,22 +1091,22 @@
       <c r="F12" s="2" t="n">
         <v>2.26</v>
       </c>
-      <c r="G12" s="2" t="n"/>
+      <c r="G12" s="2" t="n">
+        <v>2.67</v>
+      </c>
       <c r="H12" s="2" t="n">
-        <v>2.67</v>
+        <v>43.6</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>43.6</v>
+        <v>2.45</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>2.45</v>
+        <v>0.3892</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>0.3892</v>
-      </c>
-      <c r="L12" s="2" t="n">
         <v>1.3711</v>
       </c>
+      <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="n"/>
@@ -1144,18 +1139,18 @@
       <c r="F13" s="3" t="n">
         <v>2.24</v>
       </c>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n">
+      <c r="G13" s="3" t="n">
         <v>2.68</v>
       </c>
+      <c r="H13" s="3" t="n"/>
       <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
+      <c r="J13" s="3" t="n">
+        <v>0.4723</v>
+      </c>
       <c r="K13" s="3" t="n">
-        <v>0.4723</v>
-      </c>
-      <c r="L13" s="3" t="n">
         <v>1.5694</v>
       </c>
+      <c r="L13" s="3" t="n"/>
       <c r="M13" s="3" t="n"/>
       <c r="N13" s="3" t="n"/>
       <c r="O13" s="3" t="n"/>

</xml_diff>